<commit_message>
Counting the number of operations
</commit_message>
<xml_diff>
--- a/ra/time data (version 2).xlsb.xlsx
+++ b/ra/time data (version 2).xlsb.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\uni\masters nu\RA\pythonCode\ra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9101D87-BA3A-434D-86D6-F4C78D1A24C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB37C8B-08BE-46F0-8240-22502E21D89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="12">
   <si>
     <t>n</t>
   </si>
@@ -77,6 +77,12 @@
   </si>
   <si>
     <t>Log GA</t>
+  </si>
+  <si>
+    <t>Lie time</t>
+  </si>
+  <si>
+    <t>Log Lie</t>
   </si>
 </sst>
 </file>
@@ -1750,7 +1756,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'5s 500'!$F$1</c:f>
+              <c:f>'5s 500'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1837,7 +1843,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'5s 500'!$F$2:$F$20</c:f>
+              <c:f>'5s 500'!$G$2:$G$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -1912,7 +1918,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'5s 500'!$G$1</c:f>
+              <c:f>'5s 500'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1999,7 +2005,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'5s 500'!$G$2:$G$20</c:f>
+              <c:f>'5s 500'!$H$2:$H$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -2074,7 +2080,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'5s 500'!$H$1</c:f>
+              <c:f>'5s 500'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2161,7 +2167,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'5s 500'!$H$2:$H$20</c:f>
+              <c:f>'5s 500'!$I$2:$I$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -2236,7 +2242,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>'5s 500'!$I$1</c:f>
+              <c:f>'5s 500'!$J$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2257,7 +2263,7 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>'5s 500'!$I$2:$I$20</c:f>
+              <c:f>'5s 500'!$J$2:$J$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -2324,6 +2330,102 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-245C-462D-8B8A-37780AC87CF8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'5s 500'!$K$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log Lie</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'5s 500'!$K$2:$K$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.53684997576216942</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.44022930772154567</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.29017319286849264</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.22781564618396441</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.13802894547480579</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-8.4992103573121355E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-1.5310790237490447E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>5.0492008579813841E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.10579961790988042</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.13143525328183239</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.16515757726465702</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.22186517439757919</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.22614645589887022</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.26201389364324018</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.30206711108447992</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.31286672771901264</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.3511213318611538</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.37440077139638739</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.38298821687556106</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FC3A-4514-9F6E-7E809DE67A78}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2578,7 +2680,7 @@
           <c:x val="0.13053999828968746"/>
           <c:y val="0.11762405856546715"/>
           <c:w val="6.6754456035186593E-2"/>
-          <c:h val="0.20497131901064805"/>
+          <c:h val="0.25621414876331006"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -2739,7 +2841,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$F$1</c:f>
+              <c:f>'10s 1000'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2826,7 +2928,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'10s 1000'!$F$2:$F$20</c:f>
+              <c:f>'10s 1000'!$G$2:$G$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -2901,7 +3003,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$G$1</c:f>
+              <c:f>'10s 1000'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2988,7 +3090,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'10s 1000'!$G$2:$G$20</c:f>
+              <c:f>'10s 1000'!$H$2:$H$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3063,7 +3165,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$H$1</c:f>
+              <c:f>'10s 1000'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3150,7 +3252,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'10s 1000'!$H$2:$H$20</c:f>
+              <c:f>'10s 1000'!$I$2:$I$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3217,6 +3319,198 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-C636-43B8-A58C-202C8493569F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'10s 1000'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log GA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'10s 1000'!$J$2:$J$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.60777628143370055</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.46120490272665071</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.34249640435118378</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.24652464731471119</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.17794397516037561</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.11218354360775146</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-2.9340349100993781E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.5023046653805916E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.4485272310157057E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9.8097971509004067E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.11926526151951455</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.15488565628228998</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.17623707066048502</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.22556042774196874</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.23942952274241205</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.26269545993699944</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.28833198409448535</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.31131218149471546</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.34310548640818223</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C36F-4FDB-B535-983664B76F3C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'10s 1000'!$K$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log Lie</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'10s 1000'!$K$2:$K$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.30123546559882719</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.135912384320267</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-2.3311980538496129E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.6747020341326341E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.1608573012714766</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.21826694211095099</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.27967921549377178</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.32336182565248733</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.36659034780390626</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.41891351315932263</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.44746856495927739</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.48500906800264604</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.51762528069864178</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.55606666305331165</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.60501059600619167</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.60207851360727371</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.63033024440916907</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.68628314978023908</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.68530565820887357</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C36F-4FDB-B535-983664B76F3C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3470,8 +3764,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.13053999828968746"/>
           <c:y val="0.11762405856546715"/>
-          <c:w val="0.10201027786493486"/>
-          <c:h val="0.1965019209542527"/>
+          <c:w val="6.6754456035186593E-2"/>
+          <c:h val="0.25621414876331006"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -4532,7 +4826,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$F$1</c:f>
+              <c:f>'10s 1000'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4619,7 +4913,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'20s 2000'!$E$2:$E$20</c:f>
+              <c:f>'20s 2000'!$G$2:$G$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -4694,7 +4988,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$G$1</c:f>
+              <c:f>'10s 1000'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4781,7 +5075,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'20s 2000'!$F$2:$F$20</c:f>
+              <c:f>'20s 2000'!$H$2:$H$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -4856,7 +5150,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$H$1</c:f>
+              <c:f>'10s 1000'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4943,7 +5237,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'20s 2000'!$G$2:$G$20</c:f>
+              <c:f>'20s 2000'!$I$2:$I$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -5010,6 +5304,198 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-74DD-4CF3-8994-6CA467525292}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'20s 2000'!$J$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log GA</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'20s 2000'!$J$2:$J$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-0.32841833508725149</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.18216957354576901</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-6.605557688868062E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.684997800495099E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.12159004346383795</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.16825434025221242</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.22341735584863226</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.28038790367280952</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.31210467166042133</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.35643241134701598</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.38974899477887986</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.43222215886970855</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.45733947690897603</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.49420751347150244</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.51683031634136212</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.53805477121122725</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.56571277693676114</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.59174450264821588</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.60742728110436339</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2787-406C-A2D9-29895E6E4A8F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'20s 2000'!$K$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Log Lie</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'20s 2000'!$K$2:$K$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>-2.6024306353061998E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.17159608727788439</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.34175857138459592</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.40278349464472762</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.4753542992560702</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.53347248504732925</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.63297113601708699</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.65375545731044626</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.70502884262178012</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.73904630816228445</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.76877323681077103</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.79961809901103553</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.82639996751505795</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.85345958230618457</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.88589953584870018</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.90947412599277955</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.93581709644729338</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.95929807994675997</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.0037336165928343</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-2787-406C-A2D9-29895E6E4A8F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5263,8 +5749,8 @@
           <c:yMode val="edge"/>
           <c:x val="0.13053999828968746"/>
           <c:y val="0.11762405856546715"/>
-          <c:w val="0.10201027786493486"/>
-          <c:h val="0.1965019209542527"/>
+          <c:w val="6.6754456035186593E-2"/>
+          <c:h val="0.25621414876331006"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="1"/>
@@ -5425,7 +5911,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$F$1</c:f>
+              <c:f>'10s 1000'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5587,7 +6073,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$G$1</c:f>
+              <c:f>'10s 1000'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -5749,7 +6235,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$H$1</c:f>
+              <c:f>'10s 1000'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6318,7 +6804,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$F$1</c:f>
+              <c:f>'10s 1000'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6480,7 +6966,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$G$1</c:f>
+              <c:f>'10s 1000'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -6642,7 +7128,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$H$1</c:f>
+              <c:f>'10s 1000'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7211,7 +7697,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$F$1</c:f>
+              <c:f>'10s 1000'!$G$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7373,7 +7859,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$G$1</c:f>
+              <c:f>'10s 1000'!$H$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -7535,7 +8021,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>'10s 1000'!$H$1</c:f>
+              <c:f>'10s 1000'!$I$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -12991,16 +13477,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>400050</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>9526</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>71439</xdr:rowOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>304801</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>147639</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -13115,16 +13601,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>95251</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>147639</xdr:rowOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>571501</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>166689</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -15814,10 +16300,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{481F1702-F245-4AE8-A213-25754971C215}">
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -15834,19 +16320,25 @@
         <v>8</v>
       </c>
       <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -15863,23 +16355,30 @@
         <v>0.16077680001035299</v>
       </c>
       <c r="F2">
+        <v>0.29050260037183701</v>
+      </c>
+      <c r="G2">
         <f>LOG(B2)</f>
         <v>-0.58854865786206245</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <f>LOG(C2)</f>
         <v>-0.26568031914099305</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <f>LOG(D2)</f>
         <v>-1.0390538042661686</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <f>LOG(E2)</f>
         <v>-0.79377661948310396</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K2">
+        <f>LOG(F2)</f>
+        <v>-0.53684997576216942</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -15896,23 +16395,30 @@
         <v>0.171153699979186</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F20" si="0">LOG(B3)</f>
+        <v>0.362886399962008</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G20" si="0">LOG(B3)</f>
         <v>-0.41184038361690795</v>
       </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G20" si="1">LOG(C3)</f>
+      <c r="H3">
+        <f t="shared" ref="H3:H20" si="1">LOG(C3)</f>
         <v>0.36310406607463558</v>
       </c>
-      <c r="H3">
-        <f t="shared" ref="H3:H20" si="2">LOG(D3)</f>
+      <c r="I3">
+        <f t="shared" ref="I3:I20" si="2">LOG(D3)</f>
         <v>-0.90413354652145739</v>
       </c>
-      <c r="I3">
-        <f t="shared" ref="I3:I20" si="3">LOG(E3)</f>
+      <c r="J3">
+        <f t="shared" ref="J3:J20" si="3">LOG(E3)</f>
         <v>-0.76661370790106853</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <f t="shared" ref="K3:K20" si="4">LOG(F3)</f>
+        <v>-0.44022930772154567</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -15929,23 +16435,30 @@
         <v>0.214481299975886</v>
       </c>
       <c r="F4">
+        <v>0.51265690010040998</v>
+      </c>
+      <c r="G4">
         <f t="shared" si="0"/>
         <v>-0.2438966284148944</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <f t="shared" si="1"/>
         <v>0.89795131674577622</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <f t="shared" si="2"/>
         <v>-0.77754366332075331</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f t="shared" si="3"/>
         <v>-0.66861056674877373</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <f t="shared" si="4"/>
+        <v>-0.29017319286849264</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -15962,23 +16475,30 @@
         <v>0.261726500000804</v>
       </c>
       <c r="F5">
+        <v>0.59181279968470302</v>
+      </c>
+      <c r="G5">
         <f t="shared" si="0"/>
         <v>-0.18217030025439443</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <f t="shared" si="1"/>
         <v>1.2963492248187813</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f t="shared" si="2"/>
         <v>-0.64416550411506401</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f t="shared" si="3"/>
         <v>-0.58215230249782446</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K5">
+        <f t="shared" si="4"/>
+        <v>-0.22781564618396441</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
@@ -15995,23 +16515,30 @@
         <v>0.31769059994257898</v>
       </c>
       <c r="F6">
+        <v>0.72773130005225495</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="0"/>
         <v>3.4106829707643734E-2</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f t="shared" si="1"/>
         <v>1.635410352888679</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f t="shared" si="2"/>
         <v>-0.44903824770182388</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f t="shared" si="3"/>
         <v>-0.49799563519949192</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K6">
+        <f t="shared" si="4"/>
+        <v>-0.13802894547480579</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
@@ -16028,23 +16555,30 @@
         <v>0.38544899993576098</v>
       </c>
       <c r="F7">
+        <v>0.82225760025903505</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="0"/>
         <v>6.8482713761754369E-2</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <f t="shared" si="1"/>
         <v>1.9054812401049357</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f t="shared" si="2"/>
         <v>-0.41998788747057569</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f t="shared" si="3"/>
         <v>-0.4140330767873921</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K7">
+        <f t="shared" si="4"/>
+        <v>-8.4992103573121355E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -16061,23 +16595,30 @@
         <v>0.42272499995306101</v>
       </c>
       <c r="F8">
+        <v>0.96535980002954602</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="0"/>
         <v>0.13110516209373138</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <f t="shared" si="1"/>
         <v>2.1588402547316026</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f t="shared" si="2"/>
         <v>-0.39968067024833892</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f t="shared" si="3"/>
         <v>-0.37394206723934081</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K8">
+        <f t="shared" si="4"/>
+        <v>-1.5310790237490447E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
@@ -16094,23 +16635,30 @@
         <v>0.47448320011608303</v>
       </c>
       <c r="F9">
+        <v>1.1232902999036001</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="0"/>
         <v>0.21351775699630487</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <f t="shared" si="1"/>
         <v>2.3972014278122304</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <f t="shared" si="2"/>
         <v>-0.35595550718525121</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <f t="shared" si="3"/>
         <v>-0.32377915989853379</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K9">
+        <f t="shared" si="4"/>
+        <v>5.0492008579813841E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -16127,23 +16675,30 @@
         <v>0.50923950015567199</v>
       </c>
       <c r="F10">
+        <v>1.27584999985992</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="0"/>
         <v>0.24968742780530151</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <f t="shared" si="1"/>
         <v>2.5560865061967952</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <f t="shared" si="2"/>
         <v>-0.26640153903866087</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <f t="shared" si="3"/>
         <v>-0.29307791681275264</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K10">
+        <f t="shared" si="4"/>
+        <v>0.10579961790988042</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
@@ -16160,23 +16715,30 @@
         <v>0.55982999992556803</v>
       </c>
       <c r="F11">
+        <v>1.35342830000445</v>
+      </c>
+      <c r="G11">
         <f t="shared" si="0"/>
         <v>0.27664559363087632</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <f t="shared" si="1"/>
         <v>2.7808634738027793</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <f t="shared" si="2"/>
         <v>-0.31722335368556592</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <f t="shared" si="3"/>
         <v>-0.25194383246322088</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K11">
+        <f t="shared" si="4"/>
+        <v>0.13143525328183239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
@@ -16193,23 +16755,30 @@
         <v>0.61381729994900502</v>
       </c>
       <c r="F12">
+        <v>1.4627077998593401</v>
+      </c>
+      <c r="G12">
         <f t="shared" si="0"/>
         <v>0.3280124388555864</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <f t="shared" si="1"/>
         <v>2.9578717096022213</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <f t="shared" si="2"/>
         <v>-0.21218543293697692</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <f t="shared" si="3"/>
         <v>-0.21196087548954762</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K12">
+        <f t="shared" si="4"/>
+        <v>0.16515757726465702</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
@@ -16226,23 +16795,30 @@
         <v>0.67912780004553497</v>
       </c>
       <c r="F13">
+        <v>1.66672970028594</v>
+      </c>
+      <c r="G13">
         <f t="shared" si="0"/>
         <v>0.3802293369380374</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <f t="shared" si="1"/>
         <v>3.0642572313915459</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <f t="shared" si="2"/>
         <v>-0.21645371772965016</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <f t="shared" si="3"/>
         <v>-0.16804849135734951</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K13">
+        <f t="shared" si="4"/>
+        <v>0.22186517439757919</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>14</v>
       </c>
@@ -16259,23 +16835,30 @@
         <v>0.70740539999678698</v>
       </c>
       <c r="F14">
+        <v>1.68324160017073</v>
+      </c>
+      <c r="G14">
         <f t="shared" si="0"/>
         <v>0.34161255871200186</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <f t="shared" si="1"/>
         <v>3.3825190202340627</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <f t="shared" si="2"/>
         <v>-0.19681611146465802</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <f t="shared" si="3"/>
         <v>-0.15033162931084057</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <f t="shared" si="4"/>
+        <v>0.22614645589887022</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -16292,23 +16875,30 @@
         <v>0.75723750004544799</v>
       </c>
       <c r="F15">
+        <v>1.82815870037302</v>
+      </c>
+      <c r="G15">
         <f t="shared" si="0"/>
         <v>0.40898576821169425</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <f t="shared" si="1"/>
         <v>3.3818388011015577</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <f t="shared" si="2"/>
         <v>1.8866863150906826E-2</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <f t="shared" si="3"/>
         <v>-0.12076788696980725</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <f t="shared" si="4"/>
+        <v>0.26201389364324018</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>16</v>
       </c>
@@ -16325,23 +16915,30 @@
         <v>0.83966110018081896</v>
       </c>
       <c r="F16">
+        <v>2.0047818003222302</v>
+      </c>
+      <c r="G16">
         <f t="shared" si="0"/>
         <v>0.44805671088621207</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <f t="shared" si="1"/>
         <v>3.5141481507647532</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <f t="shared" si="2"/>
         <v>-7.8001568691729029E-2</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <f t="shared" si="3"/>
         <v>-7.5895966342748949E-2</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <f t="shared" si="4"/>
+        <v>0.30206711108447992</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>17</v>
       </c>
@@ -16358,23 +16955,30 @@
         <v>0.85300270002335299</v>
       </c>
       <c r="F17">
+        <v>2.0552598000504001</v>
+      </c>
+      <c r="G17">
         <f t="shared" si="0"/>
         <v>0.41308172370882884</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <f t="shared" si="1"/>
         <v>3.6022549457863358</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <f t="shared" si="2"/>
         <v>-0.12355121312165876</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <f t="shared" si="3"/>
         <v>-6.9049594150897398E-2</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <f t="shared" si="4"/>
+        <v>0.31286672771901264</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>18</v>
       </c>
@@ -16391,23 +16995,30 @@
         <v>0.92503829998895504</v>
       </c>
       <c r="F18">
+        <v>2.24450890021398</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="0"/>
         <v>0.44745263122699308</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <f t="shared" si="1"/>
         <v>3.7558622660472802</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <f t="shared" si="2"/>
         <v>-9.2481153893370735E-2</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <f t="shared" si="3"/>
         <v>-3.3840285499332941E-2</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <f t="shared" si="4"/>
+        <v>0.3511213318611538</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>19</v>
       </c>
@@ -16424,23 +17035,30 @@
         <v>0.95268479990772903</v>
       </c>
       <c r="F19">
+        <v>2.3681040001101699</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>0.48208714182648593</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <f t="shared" si="1"/>
         <v>3.8363828841125054</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <f t="shared" si="2"/>
         <v>-8.4178212379601269E-2</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <f t="shared" si="3"/>
         <v>-2.1050763898457017E-2</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <f t="shared" si="4"/>
+        <v>0.37440077139638739</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>20</v>
       </c>
@@ -16457,24 +17075,31 @@
         <v>1.0217685999814401</v>
       </c>
       <c r="F20">
+        <v>2.41539529990404</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="0"/>
         <v>0.52937901628761841</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <f t="shared" si="1"/>
         <v>3.8922811035562344</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <f t="shared" si="2"/>
         <v>-6.5905731644519627E-2</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <f t="shared" si="3"/>
         <v>9.3525522273099487E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I23" t="s">
+      <c r="K20">
+        <f t="shared" si="4"/>
+        <v>0.38298821687556106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="J23" t="s">
         <v>7</v>
       </c>
     </row>
@@ -16486,10 +17111,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4F1C10-2E17-488D-A0AD-547086CFA133}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -16506,19 +17131,25 @@
         <v>8</v>
       </c>
       <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -16535,23 +17166,30 @@
         <v>0.24673099978826901</v>
       </c>
       <c r="F2">
+        <v>0.49976349994540198</v>
+      </c>
+      <c r="G2">
         <f>LOG(B2)</f>
         <v>-0.28050298338941837</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <f>LOG(C2)</f>
         <v>4.9101678208557098E-2</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <f>LOG(D2)</f>
         <v>-0.76776647888526639</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <f>LOG(E2)</f>
         <v>-0.60777628143370055</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K2">
+        <f>LOG(F2)</f>
+        <v>-0.30123546559882719</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -16568,23 +17206,30 @@
         <v>0.34577620006166399</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F20" si="0">LOG(B3)</f>
+        <v>0.731286600232124</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G20" si="0">LOG(B3)</f>
         <v>-0.11599807523121287</v>
       </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G20" si="1">LOG(C3)</f>
+      <c r="H3">
+        <f t="shared" ref="H3:H20" si="1">LOG(C3)</f>
         <v>0.67105244589460922</v>
       </c>
-      <c r="H3">
-        <f t="shared" ref="H3:H20" si="2">LOG(D3)</f>
+      <c r="I3">
+        <f t="shared" ref="I3:I20" si="2">LOG(D3)</f>
         <v>-0.59209945985736478</v>
       </c>
-      <c r="I3">
-        <f t="shared" ref="I3:I20" si="3">LOG(E3)</f>
+      <c r="J3">
+        <f t="shared" ref="J3:J20" si="3">LOG(E3)</f>
         <v>-0.46120490272665071</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <f t="shared" ref="K3:K20" si="4">LOG(F3)</f>
+        <v>-0.135912384320267</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -16601,23 +17246,30 @@
         <v>0.45446829986758502</v>
       </c>
       <c r="F4">
+        <v>0.94773740042000998</v>
+      </c>
+      <c r="G4">
         <f t="shared" si="0"/>
         <v>1.7617573339673596E-2</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <f t="shared" si="1"/>
         <v>1.1409100977860087</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <f t="shared" si="2"/>
         <v>-0.45917018588892017</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <f t="shared" si="3"/>
         <v>-0.34249640435118378</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <f t="shared" si="4"/>
+        <v>-2.3311980538496129E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -16634,23 +17286,30 @@
         <v>0.56685939989984002</v>
       </c>
       <c r="F5">
+        <v>1.19329280033707</v>
+      </c>
+      <c r="G5">
         <f t="shared" si="0"/>
         <v>0.12531857812352648</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <f t="shared" si="1"/>
         <v>1.5271966790930642</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <f t="shared" si="2"/>
         <v>-0.37986394502624249</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <f t="shared" si="3"/>
         <v>-0.24652464731471119</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K5">
+        <f t="shared" si="4"/>
+        <v>7.6747020341326341E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
@@ -16667,23 +17326,30 @@
         <v>0.66382870008237604</v>
       </c>
       <c r="F6">
+        <v>1.4482959001325</v>
+      </c>
+      <c r="G6">
         <f t="shared" si="0"/>
         <v>0.20319612493503247</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f t="shared" si="1"/>
         <v>1.8585053160566041</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <f t="shared" si="2"/>
         <v>-0.29782804914228878</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f t="shared" si="3"/>
         <v>-0.17794397516037561</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K6">
+        <f t="shared" si="4"/>
+        <v>0.1608573012714766</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
@@ -16700,23 +17366,30 @@
         <v>0.77235410013236105</v>
       </c>
       <c r="F7">
+        <v>1.65297750011086</v>
+      </c>
+      <c r="G7">
         <f t="shared" si="0"/>
         <v>0.27535743108759814</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <f t="shared" si="1"/>
         <v>2.1812606136527593</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <f t="shared" si="2"/>
         <v>-0.22966355890485077</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f t="shared" si="3"/>
         <v>-0.11218354360775146</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K7">
+        <f t="shared" si="4"/>
+        <v>0.21826694211095099</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -16733,23 +17406,30 @@
         <v>0.9346729000099</v>
       </c>
       <c r="F8">
+        <v>1.90405380027368</v>
+      </c>
+      <c r="G8">
         <f t="shared" si="0"/>
         <v>0.34543254749914665</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <f t="shared" si="1"/>
         <v>2.4659724668498528</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <f t="shared" si="2"/>
         <v>-0.14182386201765568</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <f t="shared" si="3"/>
         <v>-2.9340349100993781E-2</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K8">
+        <f t="shared" si="4"/>
+        <v>0.27967921549377178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
@@ -16766,23 +17446,30 @@
         <v>1.03519709990359</v>
       </c>
       <c r="F9">
+        <v>2.1055319001898098</v>
+      </c>
+      <c r="G9">
         <f t="shared" si="0"/>
         <v>0.40418349821266247</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <f t="shared" si="1"/>
         <v>2.6833771387458261</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <f t="shared" si="2"/>
         <v>-0.10623823794205658</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <f t="shared" si="3"/>
         <v>1.5023046653805916E-2</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K9">
+        <f t="shared" si="4"/>
+        <v>0.32336182565248733</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -16799,23 +17486,30 @@
         <v>1.08264300017617</v>
       </c>
       <c r="F10">
+        <v>2.3258962999097998</v>
+      </c>
+      <c r="G10">
         <f t="shared" si="0"/>
         <v>0.44966349415333057</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <f t="shared" si="1"/>
         <v>2.8452488381001197</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <f t="shared" si="2"/>
         <v>-6.7678468010706816E-2</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <f t="shared" si="3"/>
         <v>3.4485272310157057E-2</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K10">
+        <f t="shared" si="4"/>
+        <v>0.36659034780390626</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
@@ -16832,23 +17526,30 @@
         <v>1.25342390011064</v>
       </c>
       <c r="F11">
+        <v>2.6236959998495801</v>
+      </c>
+      <c r="G11">
         <f t="shared" si="0"/>
         <v>0.49590494359435922</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <f t="shared" si="1"/>
         <v>3.10556372742424</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <f t="shared" si="2"/>
         <v>-1.7050711425501325E-2</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <f t="shared" si="3"/>
         <v>9.8097971509004067E-2</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K11">
+        <f t="shared" si="4"/>
+        <v>0.41891351315932263</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
@@ -16865,23 +17566,30 @@
         <v>1.3160284000914499</v>
       </c>
       <c r="F12">
+        <v>2.8020028001628798</v>
+      </c>
+      <c r="G12">
         <f t="shared" si="0"/>
         <v>0.54841398855423695</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <f t="shared" si="1"/>
         <v>3.2405537659200929</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <f t="shared" si="2"/>
         <v>1.5401673702949125E-2</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <f t="shared" si="3"/>
         <v>0.11926526151951455</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K12">
+        <f t="shared" si="4"/>
+        <v>0.44746856495927739</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
@@ -16898,23 +17606,30 @@
         <v>1.4285178000573</v>
       </c>
       <c r="F13">
+        <v>3.0549849001690701</v>
+      </c>
+      <c r="G13">
         <f t="shared" si="0"/>
         <v>0.582608730687733</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <f t="shared" si="1"/>
         <v>3.406771963700217</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <f t="shared" si="2"/>
         <v>6.3633545230784669E-2</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <f t="shared" si="3"/>
         <v>0.15488565628228998</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K13">
+        <f t="shared" si="4"/>
+        <v>0.48500906800264604</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>14</v>
       </c>
@@ -16931,23 +17646,30 @@
         <v>1.50050369999371</v>
       </c>
       <c r="F14">
+        <v>3.2932543996721502</v>
+      </c>
+      <c r="G14">
         <f t="shared" si="0"/>
         <v>0.62727366165808607</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <f t="shared" si="1"/>
         <v>3.5277273291284281</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <f t="shared" si="2"/>
         <v>9.2580300691311124E-2</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <f t="shared" si="3"/>
         <v>0.17623707066048502</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <f t="shared" si="4"/>
+        <v>0.51762528069864178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -16964,23 +17686,30 @@
         <v>1.6809717998839899</v>
       </c>
       <c r="F15">
+        <v>3.5980455996468601</v>
+      </c>
+      <c r="G15">
         <f t="shared" si="0"/>
         <v>0.6592504687726608</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <f t="shared" si="1"/>
         <v>3.6850515935762131</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <f t="shared" si="2"/>
         <v>0.11347539853673715</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <f t="shared" si="3"/>
         <v>0.22556042774196874</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <f t="shared" si="4"/>
+        <v>0.55606666305331165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>16</v>
       </c>
@@ -16997,23 +17726,30 @@
         <v>1.73551960010081</v>
       </c>
       <c r="F16">
+        <v>4.0272686001844704</v>
+      </c>
+      <c r="G16">
         <f t="shared" si="0"/>
         <v>0.68306505838291154</v>
       </c>
-      <c r="G16">
+      <c r="H16">
         <f t="shared" si="1"/>
         <v>3.925712216048606</v>
       </c>
-      <c r="H16">
+      <c r="I16">
         <f t="shared" si="2"/>
         <v>0.15048012227033458</v>
       </c>
-      <c r="I16">
+      <c r="J16">
         <f t="shared" si="3"/>
         <v>0.23942952274241205</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <f t="shared" si="4"/>
+        <v>0.60501059600619167</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>17</v>
       </c>
@@ -17030,23 +17766,30 @@
         <v>1.8310300000011901</v>
       </c>
       <c r="F17">
+        <v>4.0001706001348696</v>
+      </c>
+      <c r="G17">
         <f t="shared" si="0"/>
         <v>0.72226362737262384</v>
       </c>
-      <c r="G17">
+      <c r="H17">
         <f t="shared" si="1"/>
         <v>4.0496315590090868</v>
       </c>
-      <c r="H17">
+      <c r="I17">
         <f t="shared" si="2"/>
         <v>0.17808443287921172</v>
       </c>
-      <c r="I17">
+      <c r="J17">
         <f t="shared" si="3"/>
         <v>0.26269545993699944</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <f t="shared" si="4"/>
+        <v>0.60207851360727371</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>18</v>
       </c>
@@ -17063,23 +17806,30 @@
         <v>1.9423700999468501</v>
       </c>
       <c r="F18">
+        <v>4.2690401999279803</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="0"/>
         <v>0.75321524647887972</v>
       </c>
-      <c r="G18">
+      <c r="H18">
         <f t="shared" si="1"/>
         <v>4.1651177174029792</v>
       </c>
-      <c r="H18">
+      <c r="I18">
         <f t="shared" si="2"/>
         <v>0.19816203904607557</v>
       </c>
-      <c r="I18">
+      <c r="J18">
         <f t="shared" si="3"/>
         <v>0.28833198409448535</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <f t="shared" si="4"/>
+        <v>0.63033024440916907</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>19</v>
       </c>
@@ -17096,23 +17846,30 @@
         <v>2.0479162000119602</v>
       </c>
       <c r="F19">
+        <v>4.8560500000603497</v>
+      </c>
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>0.78015162924532189</v>
       </c>
-      <c r="G19">
+      <c r="H19">
         <f t="shared" si="1"/>
         <v>4.2150346747474483</v>
       </c>
-      <c r="H19">
+      <c r="I19">
         <f t="shared" si="2"/>
         <v>0.22549020007128417</v>
       </c>
-      <c r="I19">
+      <c r="J19">
         <f t="shared" si="3"/>
         <v>0.31131218149471546</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <f t="shared" si="4"/>
+        <v>0.68628314978023908</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>20</v>
       </c>
@@ -17129,20 +17886,27 @@
         <v>2.2034616000019001</v>
       </c>
       <c r="F20">
+        <v>4.8451324999332401</v>
+      </c>
+      <c r="G20">
         <f t="shared" si="0"/>
         <v>0.80154090619031826</v>
       </c>
-      <c r="G20">
+      <c r="H20">
         <f t="shared" si="1"/>
         <v>4.249645026330171</v>
       </c>
-      <c r="H20">
+      <c r="I20">
         <f t="shared" si="2"/>
         <v>0.24487062206524232</v>
       </c>
-      <c r="I20">
+      <c r="J20">
         <f t="shared" si="3"/>
         <v>0.34310548640818223</v>
+      </c>
+      <c r="K20">
+        <f t="shared" si="4"/>
+        <v>0.68530565820887357</v>
       </c>
     </row>
   </sheetData>
@@ -17153,10 +17917,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C72AD7-F6D4-4637-9701-4544D1141569}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -17170,16 +17934,28 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -17193,19 +17969,33 @@
         <v>0.40920000000000001</v>
       </c>
       <c r="E2">
+        <v>0.46944170002825503</v>
+      </c>
+      <c r="F2">
+        <v>0.99402560014277697</v>
+      </c>
+      <c r="G2">
         <f>LOG(B2)</f>
         <v>0.17912072960929923</v>
       </c>
-      <c r="F2">
-        <f t="shared" ref="F2:G17" si="0">LOG(C2)</f>
+      <c r="H2">
+        <f>LOG(C2)</f>
         <v>0.36068075590673898</v>
       </c>
-      <c r="G2">
-        <f t="shared" si="0"/>
+      <c r="I2">
+        <f>LOG(D2)</f>
         <v>-0.38806437495987745</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J2">
+        <f>LOG(E2)</f>
+        <v>-0.32841833508725149</v>
+      </c>
+      <c r="K2">
+        <f>LOG(F2)</f>
+        <v>-2.6024306353061998E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -17219,19 +18009,33 @@
         <v>0.59189999999999998</v>
       </c>
       <c r="E3">
-        <f>LOG(B3)</f>
+        <v>0.65740110003389396</v>
+      </c>
+      <c r="F3">
+        <v>1.4845543000847099</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G20" si="0">LOG(B3)</f>
         <v>0.26688993247105292</v>
       </c>
-      <c r="F3">
-        <f t="shared" si="0"/>
+      <c r="H3">
+        <f t="shared" ref="H3:H20" si="1">LOG(C3)</f>
         <v>0.98361730349472876</v>
       </c>
-      <c r="G3">
-        <f t="shared" si="0"/>
+      <c r="I3">
+        <f t="shared" ref="I3:I20" si="2">LOG(D3)</f>
         <v>-0.2277516600281464</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J3">
+        <f t="shared" ref="J3:J20" si="3">LOG(E3)</f>
+        <v>-0.18216957354576901</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:K20" si="4">LOG(F3)</f>
+        <v>0.17159608727788439</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -17245,19 +18049,33 @@
         <v>0.81850000000000001</v>
       </c>
       <c r="E4">
-        <f t="shared" ref="E4:E10" si="1">LOG(B4)</f>
+        <v>0.85890360013581801</v>
+      </c>
+      <c r="F4">
+        <v>2.19663840020075</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
         <v>0.40859607646278268</v>
       </c>
-      <c r="F4">
-        <f t="shared" si="0"/>
+      <c r="H4">
+        <f t="shared" si="1"/>
         <v>1.4609198138946675</v>
       </c>
-      <c r="G4">
-        <f t="shared" si="0"/>
+      <c r="I4">
+        <f t="shared" si="2"/>
         <v>-8.6981316252039753E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J4">
+        <f t="shared" si="3"/>
+        <v>-6.605557688868062E-2</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="4"/>
+        <v>0.34175857138459592</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -17271,19 +18089,33 @@
         <v>0.9778</v>
       </c>
       <c r="E5">
+        <v>1.0885540000163001</v>
+      </c>
+      <c r="F5">
+        <v>2.52803739998489</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>0.53064785352748556</v>
+      </c>
+      <c r="H5">
         <f t="shared" si="1"/>
-        <v>0.53064785352748556</v>
-      </c>
-      <c r="F5">
-        <f t="shared" si="0"/>
         <v>1.8612580333896194</v>
       </c>
-      <c r="G5">
-        <f t="shared" si="0"/>
+      <c r="I5">
+        <f t="shared" si="2"/>
         <v>-9.7499670721832143E-3</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <f t="shared" si="3"/>
+        <v>3.684997800495099E-2</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="4"/>
+        <v>0.40278349464472762</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>6</v>
       </c>
@@ -17297,19 +18129,33 @@
         <v>2.0078</v>
       </c>
       <c r="E6">
+        <v>1.32309199986048</v>
+      </c>
+      <c r="F6">
+        <v>2.9878191002644598</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>0.77826704680664749</v>
+      </c>
+      <c r="H6">
         <f t="shared" si="1"/>
-        <v>0.77826704680664749</v>
-      </c>
-      <c r="F6">
-        <f t="shared" si="0"/>
         <v>2.1768526827455936</v>
       </c>
-      <c r="G6">
-        <f t="shared" si="0"/>
+      <c r="I6">
+        <f t="shared" si="2"/>
         <v>0.30272044989613406</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <f t="shared" si="3"/>
+        <v>0.12159004346383795</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="4"/>
+        <v>0.4753542992560702</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>7</v>
       </c>
@@ -17323,19 +18169,33 @@
         <v>2.0775999999999999</v>
       </c>
       <c r="E7">
+        <v>1.47317500016652</v>
+      </c>
+      <c r="F7">
+        <v>3.4156431001611001</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>0.84486221613752133</v>
+      </c>
+      <c r="H7">
         <f t="shared" si="1"/>
-        <v>0.84486221613752133</v>
-      </c>
-      <c r="F7">
-        <f t="shared" si="0"/>
         <v>2.464359288292099</v>
       </c>
-      <c r="G7">
-        <f t="shared" si="0"/>
+      <c r="I7">
+        <f t="shared" si="2"/>
         <v>0.31756193662124627</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J7">
+        <f t="shared" si="3"/>
+        <v>0.16825434025221242</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="4"/>
+        <v>0.53347248504732925</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8</v>
       </c>
@@ -17349,19 +18209,33 @@
         <v>2.4805999999999999</v>
       </c>
       <c r="E8">
+        <v>1.6726972998585501</v>
+      </c>
+      <c r="F8">
+        <v>4.2950787995941901</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>0.91882162594644479</v>
+      </c>
+      <c r="H8">
         <f t="shared" si="1"/>
-        <v>0.91882162594644479</v>
-      </c>
-      <c r="F8">
-        <f>LOG(C8)</f>
         <v>2.7060008232242336</v>
       </c>
-      <c r="G8">
-        <f t="shared" si="0"/>
+      <c r="I8">
+        <f t="shared" si="2"/>
         <v>0.39455673936365637</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J8">
+        <f t="shared" si="3"/>
+        <v>0.22341735584863226</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="4"/>
+        <v>0.63297113601708699</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9</v>
       </c>
@@ -17375,19 +18249,33 @@
         <v>2.7888999999999999</v>
       </c>
       <c r="E9">
+        <v>1.9071633999701501</v>
+      </c>
+      <c r="F9">
+        <v>4.5056292996741796</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>0.96270546410180979</v>
+      </c>
+      <c r="H9">
         <f t="shared" si="1"/>
-        <v>0.96270546410180979</v>
-      </c>
-      <c r="F9">
-        <f t="shared" si="0"/>
         <v>2.9274268362844258</v>
       </c>
-      <c r="G9">
-        <f t="shared" si="0"/>
+      <c r="I9">
+        <f t="shared" si="2"/>
         <v>0.44543294229516656</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J9">
+        <f t="shared" si="3"/>
+        <v>0.28038790367280952</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="4"/>
+        <v>0.65375545731044626</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>10</v>
       </c>
@@ -17401,19 +18289,33 @@
         <v>3.2602000000000002</v>
       </c>
       <c r="E10">
+        <v>2.0516566000878802</v>
+      </c>
+      <c r="F10">
+        <v>5.0702437995932996</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>1.0239640369866647</v>
+      </c>
+      <c r="H10">
         <f t="shared" si="1"/>
-        <v>1.0239640369866647</v>
-      </c>
-      <c r="F10">
-        <f t="shared" si="0"/>
         <v>3.1256414735043663</v>
       </c>
-      <c r="G10">
-        <f t="shared" si="0"/>
+      <c r="I10">
+        <f t="shared" si="2"/>
         <v>0.51324424308392258</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J10">
+        <f t="shared" si="3"/>
+        <v>0.31210467166042133</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="4"/>
+        <v>0.70502884262178012</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>11</v>
       </c>
@@ -17427,19 +18329,33 @@
         <v>3.6480999999999999</v>
       </c>
       <c r="E11">
-        <f>LOG(B11)</f>
+        <v>2.2721259999088899</v>
+      </c>
+      <c r="F11">
+        <v>5.4833542997948799</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
         <v>1.0678330862343137</v>
       </c>
-      <c r="F11">
-        <f t="shared" si="0"/>
+      <c r="H11">
+        <f t="shared" si="1"/>
         <v>3.3018647321002264</v>
       </c>
-      <c r="G11">
-        <f t="shared" si="0"/>
+      <c r="I11">
+        <f t="shared" si="2"/>
         <v>0.56206673449545508</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J11">
+        <f t="shared" si="3"/>
+        <v>0.35643241134701598</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="4"/>
+        <v>0.73904630816228445</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>12</v>
       </c>
@@ -17453,19 +18369,33 @@
         <v>3.9548999999999999</v>
       </c>
       <c r="E12">
-        <f>LOG(B12)</f>
+        <v>2.45329059986397</v>
+      </c>
+      <c r="F12">
+        <v>5.8718268000520704</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="0"/>
         <v>1.1250190736565042</v>
       </c>
-      <c r="F12">
-        <f t="shared" si="0"/>
+      <c r="H12">
+        <f t="shared" si="1"/>
         <v>3.4711752869273647</v>
       </c>
-      <c r="G12">
-        <f t="shared" si="0"/>
+      <c r="I12">
+        <f t="shared" si="2"/>
         <v>0.59713550679772964</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J12">
+        <f t="shared" si="3"/>
+        <v>0.38974899477887986</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="4"/>
+        <v>0.76877323681077103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>13</v>
       </c>
@@ -17479,19 +18409,33 @@
         <v>4.2637999999999998</v>
       </c>
       <c r="E13">
-        <f t="shared" ref="E13:E19" si="2">LOG(B13)</f>
+        <v>2.7053419000003398</v>
+      </c>
+      <c r="F13">
+        <v>6.3040275000966997</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
         <v>1.2045784641095207</v>
       </c>
-      <c r="F13">
-        <f t="shared" ref="F13:F20" si="3">LOG(C13)</f>
+      <c r="H13">
+        <f t="shared" si="1"/>
         <v>3.6268820043517778</v>
       </c>
-      <c r="G13">
-        <f t="shared" si="0"/>
+      <c r="I13">
+        <f t="shared" si="2"/>
         <v>0.62979682525550629</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="J13">
+        <f t="shared" si="3"/>
+        <v>0.43222215886970855</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="4"/>
+        <v>0.79961809901103553</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>14</v>
       </c>
@@ -17505,19 +18449,33 @@
         <v>4.7336999999999998</v>
       </c>
       <c r="E14">
+        <v>2.8664176999591202</v>
+      </c>
+      <c r="F14">
+        <v>6.7050183000974304</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>1.2068987019193613</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="1"/>
+        <v>3.7693818979616709</v>
+      </c>
+      <c r="I14">
         <f t="shared" si="2"/>
-        <v>1.2068987019193613</v>
-      </c>
-      <c r="F14">
+        <v>0.67520073089069388</v>
+      </c>
+      <c r="J14">
         <f t="shared" si="3"/>
-        <v>3.7693818979616709</v>
-      </c>
-      <c r="G14">
-        <f t="shared" si="0"/>
-        <v>0.67520073089069388</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.45733947690897603</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="4"/>
+        <v>0.82639996751505795</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -17531,19 +18489,33 @@
         <v>5.0602999999999998</v>
       </c>
       <c r="E15">
+        <v>3.1203801999799898</v>
+      </c>
+      <c r="F15">
+        <v>7.1360778999514798</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>1.2361844428801496</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="1"/>
+        <v>3.9046200224387309</v>
+      </c>
+      <c r="I15">
         <f t="shared" si="2"/>
-        <v>1.2361844428801496</v>
-      </c>
-      <c r="F15">
+        <v>0.70417626476122619</v>
+      </c>
+      <c r="J15">
         <f t="shared" si="3"/>
-        <v>3.9046200224387309</v>
-      </c>
-      <c r="G15">
-        <f t="shared" si="0"/>
-        <v>0.70417626476122619</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.49420751347150244</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="4"/>
+        <v>0.85345958230618457</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>16</v>
       </c>
@@ -17557,19 +18529,33 @@
         <v>5.3571</v>
       </c>
       <c r="E16">
-        <f>LOG(B16)</f>
+        <v>3.2872317000292202</v>
+      </c>
+      <c r="F16">
+        <v>7.6895254002884004</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
         <v>1.259271263185658</v>
       </c>
-      <c r="F16">
+      <c r="H16">
+        <f t="shared" si="1"/>
+        <v>4.0334210290741446</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="2"/>
+        <v>0.72892975334370924</v>
+      </c>
+      <c r="J16">
         <f t="shared" si="3"/>
-        <v>4.0334210290741446</v>
-      </c>
-      <c r="G16">
-        <f t="shared" si="0"/>
-        <v>0.72892975334370924</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.51683031634136212</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="4"/>
+        <v>0.88589953584870018</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>17</v>
       </c>
@@ -17583,19 +18569,33 @@
         <v>5.5542999999999996</v>
       </c>
       <c r="E17">
+        <v>3.4518727001268399</v>
+      </c>
+      <c r="F17">
+        <v>8.1184688000939698</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>1.3012145316076791</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="1"/>
+        <v>4.1832130896040161</v>
+      </c>
+      <c r="I17">
         <f t="shared" si="2"/>
-        <v>1.3012145316076791</v>
-      </c>
-      <c r="F17">
+        <v>0.74462933325109992</v>
+      </c>
+      <c r="J17">
         <f t="shared" si="3"/>
-        <v>4.1832130896040161</v>
-      </c>
-      <c r="G17">
-        <f t="shared" si="0"/>
-        <v>0.74462933325109992</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.53805477121122725</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="4"/>
+        <v>0.90947412599277955</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>18</v>
       </c>
@@ -17609,19 +18609,33 @@
         <v>5.9537000000000004</v>
       </c>
       <c r="E18">
+        <v>3.6788558999542098</v>
+      </c>
+      <c r="F18">
+        <v>8.6261518001556396</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>1.3255505532952461</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="1"/>
+        <v>4.2754123710177439</v>
+      </c>
+      <c r="I18">
         <f t="shared" si="2"/>
-        <v>1.3255505532952461</v>
-      </c>
-      <c r="F18">
+        <v>0.774786947269548</v>
+      </c>
+      <c r="J18">
         <f t="shared" si="3"/>
-        <v>4.2754123710177439</v>
-      </c>
-      <c r="G18">
-        <f t="shared" ref="G18:G20" si="4">LOG(D18)</f>
-        <v>0.774786947269548</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.56571277693676114</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="4"/>
+        <v>0.93581709644729338</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>19</v>
       </c>
@@ -17635,19 +18649,33 @@
         <v>6.1835000000000004</v>
       </c>
       <c r="E19">
+        <v>3.9061102999839901</v>
+      </c>
+      <c r="F19">
+        <v>9.1053801001980901</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>1.3520956505279338</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="1"/>
+        <v>4.4002371006387984</v>
+      </c>
+      <c r="I19">
         <f t="shared" si="2"/>
-        <v>1.3520956505279338</v>
-      </c>
-      <c r="F19">
+        <v>0.79123436512436673</v>
+      </c>
+      <c r="J19">
         <f t="shared" si="3"/>
-        <v>4.4002371006387984</v>
-      </c>
-      <c r="G19">
+        <v>0.59174450264821588</v>
+      </c>
+      <c r="K19">
         <f t="shared" si="4"/>
-        <v>0.79123436512436673</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>0.95929807994675997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>20</v>
       </c>
@@ -17661,16 +18689,30 @@
         <v>6.6779000000000002</v>
       </c>
       <c r="E20">
-        <f>LOG(B20)</f>
+        <v>4.0497413000557501</v>
+      </c>
+      <c r="F20">
+        <v>10.0863402998074</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
         <v>1.3096110069525659</v>
       </c>
-      <c r="F20">
+      <c r="H20">
+        <f t="shared" si="1"/>
+        <v>4.5676086152707969</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="2"/>
+        <v>0.82463991130814507</v>
+      </c>
+      <c r="J20">
         <f t="shared" si="3"/>
-        <v>4.5676086152707969</v>
-      </c>
-      <c r="G20">
+        <v>0.60742728110436339</v>
+      </c>
+      <c r="K20">
         <f t="shared" si="4"/>
-        <v>0.82463991130814507</v>
+        <v>1.0037336165928343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>